<commit_message>
adding Green Manager entry
new entry
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750FB251-A1A5-4BD0-99C4-AD9A128CA12B}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DAE7252-13BA-46F9-A0C1-648531EC6612}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>source_paper</t>
   </si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t>iStar2.0 with context annotations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iStar2.0  </t>
+  </si>
+  <si>
+    <t>Smart Home</t>
   </si>
 </sst>
 </file>
@@ -559,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -759,6 +765,20 @@
         <v>41</v>
       </c>
     </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>2019</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixing green manager entry
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="102" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DAE7252-13BA-46F9-A0C1-648531EC6612}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D19B4A96-CCA3-4CEC-BADB-6F906A88AF23}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>source_paper</t>
   </si>
@@ -174,13 +174,22 @@
   </si>
   <si>
     <t>Smart Home</t>
+  </si>
+  <si>
+    <t>A. Inmaculada, A. Mercedes, J.M. Horcas, L. Fuentes</t>
+  </si>
+  <si>
+    <t>A goal-driven software product line approach for evolving on multi-agent systems in the Internet of Things, DOI: 10.1016/j.knosys.2019.104883</t>
+  </si>
+  <si>
+    <t>GreenManager_MultiAgentSmartHome</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,6 +201,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -220,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -230,6 +245,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -766,6 +784,15 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="D9">
         <v>2019</v>
       </c>

</xml_diff>

<commit_message>
education Search system entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB167A6C-0564-4304-9D7E-195BA1B3012B}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9B18DA9-10D8-42FA-8122-6F1F00D67754}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="102">
   <si>
     <t>source_paper</t>
   </si>
@@ -336,6 +336,18 @@
   </si>
   <si>
     <t>Can goal reasoning techniques be used for strategic decision-making?</t>
+  </si>
+  <si>
+    <t>10.1007/978-3-319-46397-1_41</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> E. Paja, A. Mate, C. Woo, J. Mylopoulos</t>
+  </si>
+  <si>
+    <t>Travel &amp; Hospitality</t>
+  </si>
+  <si>
+    <t>iStar 1.0 with satisfaction annotations</t>
   </si>
 </sst>
 </file>
@@ -1204,6 +1216,24 @@
       <c r="B18" s="4" t="s">
         <v>97</v>
       </c>
+      <c r="C18" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18">
+        <v>2016</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>

</xml_diff>

<commit_message>
update on png file
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9B18DA9-10D8-42FA-8122-6F1F00D67754}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C1846F7-92E6-4C92-9AAD-500851DA450E}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="107">
   <si>
     <t>source_paper</t>
   </si>
@@ -348,6 +348,21 @@
   </si>
   <si>
     <t>iStar 1.0 with satisfaction annotations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SearchSystem_inEducation </t>
+  </si>
+  <si>
+    <t>A design framework for generating BDI-agents from goal models</t>
+  </si>
+  <si>
+    <t> 10.1145/1329125.1329307</t>
+  </si>
+  <si>
+    <t>L. Penserini, A. Perini, A. Susi, M. Morandini, J. Mylopoulos</t>
+  </si>
+  <si>
+    <t>Education</t>
   </si>
 </sst>
 </file>
@@ -759,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -1210,30 +1225,62 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>96</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" t="s">
         <v>98</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" t="s">
         <v>99</v>
       </c>
       <c r="E18">
         <v>2016</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" t="s">
         <v>100</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="4" t="s">
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
         <v>101</v>
       </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19">
+        <v>2007</v>
+      </c>
+      <c r="F19" t="s">
+        <v>106</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>

</xml_diff>

<commit_message>
Pizza buisiness entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DAF4C17-8ABE-46FD-81C9-410E00B20926}"/>
+  <xr:revisionPtr revIDLastSave="265" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6DA71C3-5567-4BB1-BB1C-14627D9BAE15}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="128">
   <si>
     <t>source_paper</t>
   </si>
@@ -423,13 +423,16 @@
   </si>
   <si>
     <t>E. Cardoso, J. Almeida, G. Guizzardi, R. Guizzardi</t>
+  </si>
+  <si>
+    <t>PizzaCompany_andDelivery</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,6 +458,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF800000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -484,7 +494,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -499,6 +509,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -834,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -1440,6 +1453,11 @@
         <v>8</v>
       </c>
     </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Course manager entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6DA71C3-5567-4BB1-BB1C-14627D9BAE15}"/>
+  <xr:revisionPtr revIDLastSave="273" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F2818BE-7F66-422E-92C3-6EBFAAC4D424}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="132">
   <si>
     <t>source_paper</t>
   </si>
@@ -426,13 +426,25 @@
   </si>
   <si>
     <t>PizzaCompany_andDelivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methodology of synchronization among strategy and operation. A standards-based modeling approach </t>
+  </si>
+  <si>
+    <t>10.15446/ing.investig.v37n2.60869</t>
+  </si>
+  <si>
+    <t> V. Collazos, H. Duarte</t>
+  </si>
+  <si>
+    <t>Food Delivery Business</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -458,13 +470,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF800000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -494,7 +499,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -509,9 +514,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1454,8 +1456,29 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" t="s">
         <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" t="s">
+        <v>130</v>
+      </c>
+      <c r="E24">
+        <v>2017</v>
+      </c>
+      <c r="F24" t="s">
+        <v>131</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
smart city entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BFE6480-8DE7-4F9B-9FA1-E4F8222C5764}"/>
+  <xr:revisionPtr revIDLastSave="300" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D642DD1-D36E-4577-B706-122608A703E0}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="147">
   <si>
     <t>source_paper</t>
   </si>
@@ -468,6 +468,21 @@
   </si>
   <si>
     <t>Construction industry</t>
+  </si>
+  <si>
+    <t>SmartCity_monolithicCaseStudy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improving Requirements in Model-Based Systems Engineering Through Multi-layer Goal Models </t>
+  </si>
+  <si>
+    <t>10.1007/978-3-031-66339-0_8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Ponsard, R. Darimont </t>
+  </si>
+  <si>
+    <t>Smart City</t>
   </si>
 </sst>
 </file>
@@ -879,7 +894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -1563,6 +1578,32 @@
         <v>23</v>
       </c>
     </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E27" s="4">
+        <v>2024</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>
   <hyperlinks>

</xml_diff>

<commit_message>
telemedicinen case study entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="329" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57448A2D-105A-414E-8B5B-630081D55178}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DB7D9A0-5337-4675-925A-6458CCF73202}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="168">
   <si>
     <t>source_paper</t>
   </si>
@@ -531,6 +531,21 @@
   </si>
   <si>
     <t>Aeronautics</t>
+  </si>
+  <si>
+    <t>PatientAndProvider_remoteHealthcare</t>
+  </si>
+  <si>
+    <t>Sensitivity Analysis of Conflicting Goals in the i* Goal Model</t>
+  </si>
+  <si>
+    <t>10.1093/comjnl/bxaa189</t>
+  </si>
+  <si>
+    <t> S. Sumesh, A. Krishna</t>
+  </si>
+  <si>
+    <t>Telemedicine</t>
   </si>
 </sst>
 </file>
@@ -942,7 +957,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -1730,6 +1745,50 @@
         <v>23</v>
       </c>
     </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>163</v>
+      </c>
+      <c r="B31" t="s">
+        <v>164</v>
+      </c>
+      <c r="C31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" t="s">
+        <v>166</v>
+      </c>
+      <c r="E31">
+        <v>2022</v>
+      </c>
+      <c r="F31" t="s">
+        <v>167</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>
   <hyperlinks>

</xml_diff>

<commit_message>
SD model entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="338" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DB7D9A0-5337-4675-925A-6458CCF73202}"/>
+  <xr:revisionPtr revIDLastSave="348" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E65ED13-93B2-4FB0-B8B2-3DCCF351B957}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="172">
   <si>
     <t>source_paper</t>
   </si>
@@ -546,6 +546,18 @@
   </si>
   <si>
     <t>Telemedicine</t>
+  </si>
+  <si>
+    <t>ValidationAndVerification_RE_SDView</t>
+  </si>
+  <si>
+    <t> Requirements engineering for distributed development using software agents</t>
+  </si>
+  <si>
+    <t>10.1007/978-3-540-87991-6_33</t>
+  </si>
+  <si>
+    <t>M. Sayao, A. Haendchen, H. Do Prado</t>
   </si>
 </sst>
 </file>
@@ -1772,7 +1784,30 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32"/>
+      <c r="A32" t="s">
+        <v>168</v>
+      </c>
+      <c r="B32" t="s">
+        <v>169</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" t="s">
+        <v>171</v>
+      </c>
+      <c r="E32">
+        <v>2008</v>
+      </c>
+      <c r="F32" t="s">
+        <v>35</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33"/>

</xml_diff>

<commit_message>
business strategy models entry
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="428" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B93BBC9-FE48-445A-8AFB-DF03F72EBE47}"/>
+  <xr:revisionPtr revIDLastSave="451" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9AFC844-4E51-478A-AE20-8859EE7A7475}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="214">
   <si>
     <t>source_paper</t>
   </si>
@@ -663,6 +663,27 @@
   </si>
   <si>
     <t>reconstructed-from-author</t>
+  </si>
+  <si>
+    <t>Software Product Lines (SPL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Including business strategy in model-driven methods: an experiment </t>
+  </si>
+  <si>
+    <t>10.1007/s00766-023-00400-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> R. Noel, J. Panach, O. Pastor </t>
+  </si>
+  <si>
+    <t>BusinessStrategy_TelecommunicationsCompany</t>
+  </si>
+  <si>
+    <t>Business Strategy; Telecommunication</t>
+  </si>
+  <si>
+    <t>Business Strategy; Insurance</t>
   </si>
 </sst>
 </file>
@@ -1074,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -2136,12 +2157,67 @@
         <v>205</v>
       </c>
       <c r="E41">
-        <v>2023</v>
+        <v>2017</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>207</v>
       </c>
       <c r="G41" s="4" t="s">
         <v>206</v>
       </c>
       <c r="H41" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E42">
+        <v>2023</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E43">
+        <v>2023</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" s="4" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
smart home entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="517" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39C9AD1C-7369-4BB2-BC95-07D55FC98E99}"/>
+  <xr:revisionPtr revIDLastSave="527" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDDDFE44-1032-4FA2-B328-5AF3D98B92DF}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="253">
   <si>
     <t>source_paper</t>
   </si>
@@ -788,7 +788,19 @@
     <t>iStar 1.0 with context and task annotations</t>
   </si>
   <si>
-    <t> TaRGeT_MotorolaProject</t>
+    <t>Goals and Scenarios for Requirements Engineering of Software Product Lines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ceur-ws.org/Vol-766/ </t>
+  </si>
+  <si>
+    <t>G. Guedes, C. Silva, J. Castro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iStar 1.0 with context and cardinality annotations </t>
+  </si>
+  <si>
+    <t>TaRGeT_MotorolaProject</t>
   </si>
 </sst>
 </file>
@@ -2530,9 +2542,30 @@
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>248</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="E51" s="1">
+        <v>2011</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
museum assistance 2 entry added
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="573" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F262DAF0-0F14-4D30-887A-8BCC076C5B59}"/>
+  <xr:revisionPtr revIDLastSave="583" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D76BB822-AD67-4FDF-A1B0-625179992F54}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="287">
   <si>
     <t>source_paper</t>
   </si>
@@ -885,6 +885,24 @@
   </si>
   <si>
     <t>iStar 1.0 with dynamic functions and evaluation annotations</t>
+  </si>
+  <si>
+    <t>PatientCareGivingSystem_SmartHome</t>
+  </si>
+  <si>
+    <t>Reasoning with contextual requirements: Detecting inconsistency and conflicts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smart Home System; Healthcare </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tropos 1.0 with context annotations </t>
+  </si>
+  <si>
+    <t>MuseumGuide_MobileInformationSystem</t>
+  </si>
+  <si>
+    <t>A goal-based framework for contextual requirements modeling and analysis</t>
   </si>
 </sst>
 </file>
@@ -1296,7 +1314,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -2783,7 +2801,38 @@
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="4"/>
+      <c r="A57" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E57" s="1">
+        <v>2013</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>286</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>

</xml_diff>

<commit_message>
new entry safe flight
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="583" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D76BB822-AD67-4FDF-A1B0-625179992F54}"/>
+  <xr:revisionPtr revIDLastSave="592" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9A56724-6623-4498-8910-E67AF21A3CA6}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="292">
   <si>
     <t>source_paper</t>
   </si>
@@ -903,13 +903,28 @@
   </si>
   <si>
     <t>A goal-based framework for contextual requirements modeling and analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1007/s00766-010-0110-z </t>
+  </si>
+  <si>
+    <t xml:space="preserve">R. Ali, F. Dalpiaz, P. Giorgini </t>
+  </si>
+  <si>
+    <t>SafeFlight_ATC</t>
+  </si>
+  <si>
+    <t>From goal modeling of real-time control systems to rt-devs safety properties analysis</t>
+  </si>
+  <si>
+    <t>10.3182/20140514-3-fr-4046.00026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -935,6 +950,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF800000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -964,7 +986,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -979,6 +1001,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1314,7 +1339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -2833,6 +2858,35 @@
       <c r="B58" s="4" t="s">
         <v>286</v>
       </c>
+      <c r="C58" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="E58" s="1">
+        <v>2010</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>291</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>

</xml_diff>

<commit_message>
Eye CAre treatment entry
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="592" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9A56724-6623-4498-8910-E67AF21A3CA6}"/>
+  <xr:revisionPtr revIDLastSave="606" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66B12A6D-DCAE-40C4-88A7-940B7E734D8E}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="298">
   <si>
     <t>source_paper</t>
   </si>
@@ -704,9 +704,6 @@
     <t>DataWarehouse_inHospital</t>
   </si>
   <si>
-    <t xml:space="preserve">odel-based requirements engineering for data warehouses: From mulitdimensional modelling to KPI monitoring </t>
-  </si>
-  <si>
     <t>10.1007/978-3-319-25747-1_20</t>
   </si>
   <si>
@@ -918,6 +915,27 @@
   </si>
   <si>
     <t>10.3182/20140514-3-fr-4046.00026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N. Darragi, E. M. El-Koursi, S. Collart-Dutilleul </t>
+  </si>
+  <si>
+    <t>Air Traffic Control (ATC); Aeronautics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model-based requirements engineering for data warehouses: From mulitdimensional modelling to KPI monitoring </t>
+  </si>
+  <si>
+    <t> Aligning goal and value models for information system design</t>
+  </si>
+  <si>
+    <t>EyeCareTreatment</t>
+  </si>
+  <si>
+    <t>10.1007/978-3-642-01187-0_11</t>
+  </si>
+  <si>
+    <t>A. Edirisuriya, J. Zdravkovic</t>
   </si>
 </sst>
 </file>
@@ -1339,7 +1357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -2506,19 +2524,19 @@
         <v>219</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>222</v>
       </c>
       <c r="E45" s="1">
         <v>2015</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>15</v>
@@ -2531,16 +2549,16 @@
     </row>
     <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="C46" s="1" t="s">
-        <v>226</v>
-      </c>
       <c r="D46" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E46" s="1">
         <v>2013</v>
@@ -2559,22 +2577,22 @@
     </row>
     <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>230</v>
       </c>
       <c r="E47" s="1">
         <v>2014</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>15</v>
@@ -2587,16 +2605,16 @@
     </row>
     <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>236</v>
       </c>
       <c r="E48" s="1">
         <v>2012</v>
@@ -2615,25 +2633,25 @@
     </row>
     <row r="49" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="C49" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>239</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>240</v>
       </c>
       <c r="E49" s="1">
         <v>2019</v>
       </c>
       <c r="F49" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G49" s="1" t="s">
         <v>241</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>242</v>
       </c>
       <c r="H49" s="1" t="s">
         <v>23</v>
@@ -2643,16 +2661,16 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="C50" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="D50" s="4" t="s">
         <v>245</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>246</v>
       </c>
       <c r="E50" s="1">
         <v>2013</v>
@@ -2664,23 +2682,23 @@
         <v>15</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
     </row>
     <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B51" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C51" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="D51" s="4" t="s">
         <v>249</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>250</v>
       </c>
       <c r="E51" s="1">
         <v>2011</v>
@@ -2692,53 +2710,53 @@
         <v>15</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="C52" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="D52" s="4" t="s">
         <v>255</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>256</v>
       </c>
       <c r="E52" s="1">
         <v>2012</v>
       </c>
       <c r="F52" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H52" s="1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="C53" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>261</v>
-      </c>
       <c r="D53" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E53" s="1">
         <v>2012</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>15</v>
@@ -2749,91 +2767,91 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="C54" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="D54" s="4" t="s">
         <v>265</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>266</v>
       </c>
       <c r="E54" s="1">
         <v>2010</v>
       </c>
       <c r="F54" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H54" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="C55" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="D55" s="4" t="s">
         <v>271</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>272</v>
       </c>
       <c r="E55" s="1">
         <v>2006</v>
       </c>
       <c r="F55" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" s="4" t="s">
         <v>273</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H55" s="4" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="C56" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="D56" s="4" t="s">
         <v>277</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>278</v>
       </c>
       <c r="E56" s="1">
         <v>2016</v>
       </c>
       <c r="F56" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" s="4" t="s">
         <v>279</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H56" s="4" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B57" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>282</v>
-      </c>
       <c r="C57" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>7</v>
@@ -2842,27 +2860,27 @@
         <v>2013</v>
       </c>
       <c r="F57" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H57" s="4" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B58" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="C58" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="D58" s="4" t="s">
         <v>287</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>288</v>
       </c>
       <c r="E58" s="1">
         <v>2010</v>
@@ -2874,18 +2892,59 @@
         <v>15</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="B59" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="C59" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="D59" s="4" t="s">
         <v>291</v>
+      </c>
+      <c r="E59" s="1">
+        <v>2014</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="E60" s="1">
+        <v>2009</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished model reconstruction phase
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="658" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F372BE40-385D-4954-AA36-22FD58FF8592}"/>
+  <xr:revisionPtr revIDLastSave="659" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE1A66FB-DD28-478E-A4EC-B54F34350AB0}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
@@ -1038,7 +1038,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1064,13 +1064,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF800000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1100,7 +1093,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1115,9 +1108,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2755,17 +2745,17 @@
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="D50" s="1" t="s">
         <v>245</v>
       </c>
       <c r="E50" s="1">
@@ -2784,16 +2774,16 @@
       <c r="J50" s="1"/>
     </row>
     <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D51" s="4" t="s">
+      <c r="D51" s="1" t="s">
         <v>249</v>
       </c>
       <c r="E51" s="1">
@@ -2805,21 +2795,21 @@
       <c r="G51" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H51" s="4" t="s">
+      <c r="H51" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" s="4" t="s">
+    <row r="52" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="D52" s="4" t="s">
+      <c r="D52" s="1" t="s">
         <v>255</v>
       </c>
       <c r="E52" s="1">
@@ -2835,17 +2825,17 @@
         <v>257</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="D53" s="4" t="s">
+      <c r="D53" s="1" t="s">
         <v>255</v>
       </c>
       <c r="E53" s="1">
@@ -2861,23 +2851,23 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C54" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="D54" s="1" t="s">
         <v>265</v>
       </c>
       <c r="E54" s="1">
         <v>2010</v>
       </c>
-      <c r="F54" s="4" t="s">
+      <c r="F54" s="1" t="s">
         <v>266</v>
       </c>
       <c r="G54" s="1" t="s">
@@ -2887,43 +2877,43 @@
         <v>267</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="D55" s="4" t="s">
+      <c r="D55" s="1" t="s">
         <v>271</v>
       </c>
       <c r="E55" s="1">
         <v>2006</v>
       </c>
-      <c r="F55" s="4" t="s">
+      <c r="F55" s="1" t="s">
         <v>272</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H55" s="4" t="s">
+      <c r="H55" s="1" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="D56" s="4" t="s">
+      <c r="D56" s="1" t="s">
         <v>277</v>
       </c>
       <c r="E56" s="1">
@@ -2935,267 +2925,267 @@
       <c r="G56" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H56" s="4" t="s">
+      <c r="H56" s="1" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C57" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="D57" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E57" s="1">
         <v>2013</v>
       </c>
-      <c r="F57" s="4" t="s">
+      <c r="F57" s="1" t="s">
         <v>282</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H57" s="4" t="s">
+      <c r="H57" s="1" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="C58" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="D58" s="4" t="s">
+      <c r="D58" s="1" t="s">
         <v>287</v>
       </c>
       <c r="E58" s="1">
         <v>2010</v>
       </c>
-      <c r="F58" s="4" t="s">
+      <c r="F58" s="1" t="s">
         <v>117</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H58" s="4" t="s">
+      <c r="H58" s="1" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="6" t="s">
+    <row r="59" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="D59" s="4" t="s">
+      <c r="D59" s="1" t="s">
         <v>291</v>
       </c>
       <c r="E59" s="1">
         <v>2014</v>
       </c>
-      <c r="F59" s="4" t="s">
+      <c r="F59" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="G59" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H59" s="4" t="s">
+      <c r="G59" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="D60" s="4" t="s">
+      <c r="D60" s="1" t="s">
         <v>297</v>
       </c>
       <c r="E60" s="1">
         <v>2009</v>
       </c>
-      <c r="F60" s="4" t="s">
+      <c r="F60" s="1" t="s">
         <v>111</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H60" s="4" t="s">
+      <c r="H60" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="D61" s="4" t="s">
+      <c r="D61" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E61" s="1">
         <v>2018</v>
       </c>
-      <c r="F61" s="4" t="s">
+      <c r="F61" s="1" t="s">
         <v>302</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H61" s="4" t="s">
+      <c r="H61" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="C62" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="D62" s="4" t="s">
+      <c r="D62" s="1" t="s">
         <v>308</v>
       </c>
       <c r="E62" s="1">
         <v>2011</v>
       </c>
-      <c r="F62" s="4" t="s">
+      <c r="F62" s="1" t="s">
         <v>304</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H62" s="4" t="s">
+      <c r="H62" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="4" t="s">
+    <row r="63" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="B63" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="C63" s="4" t="s">
+      <c r="C63" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="D63" s="4" t="s">
+      <c r="D63" s="1" t="s">
         <v>312</v>
       </c>
       <c r="E63" s="1">
         <v>2013</v>
       </c>
-      <c r="F63" s="4" t="s">
+      <c r="F63" s="1" t="s">
         <v>313</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H63" s="4" t="s">
+      <c r="H63" s="1" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B64" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="C64" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="D64" s="4" t="s">
+      <c r="D64" s="1" t="s">
         <v>318</v>
       </c>
       <c r="E64" s="1">
         <v>2013</v>
       </c>
-      <c r="F64" s="4" t="s">
+      <c r="F64" s="1" t="s">
         <v>319</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H64" s="4" t="s">
+      <c r="H64" s="1" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="6" t="s">
+    <row r="65" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B65" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="C65" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="D65" s="4" t="s">
+      <c r="D65" s="1" t="s">
         <v>324</v>
       </c>
       <c r="E65" s="1">
         <v>2023</v>
       </c>
-      <c r="F65" s="4" t="s">
+      <c r="F65" s="1" t="s">
         <v>325</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H65" s="4" t="s">
+      <c r="H65" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="4" t="s">
+    <row r="66" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="B66" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="C66" s="4" t="s">
+      <c r="C66" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="D66" s="4" t="s">
+      <c r="D66" s="1" t="s">
         <v>329</v>
       </c>
       <c r="E66" s="1">
         <v>2013</v>
       </c>
-      <c r="F66" s="4" t="s">
+      <c r="F66" s="1" t="s">
         <v>122</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H66" s="4" t="s">
+      <c r="H66" s="1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adjustments for metadata field reconstrucotr
</commit_message>
<xml_diff>
--- a/metadata_catalogue.xlsx
+++ b/metadata_catalogue.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/633d15f4b43630ba/Dokumente/GitHub/GoalModelRepository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="694" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2714653-9127-402B-A481-283C7461235F}"/>
+  <xr:revisionPtr revIDLastSave="708" documentId="8_{EFB9F745-292C-44B3-BAD5-6074C357DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F06D4097-3FB8-47AC-9BF6-E1A4D7FA916B}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{25083A1C-6D06-4C71-AE29-A2B728AD67F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="346">
   <si>
     <t>source_paper</t>
   </si>
@@ -1071,35 +1071,25 @@
   </si>
   <si>
     <t>10.1007/978-3-031-72107-6_5</t>
+  </si>
+  <si>
+    <t>Reconstructor</t>
+  </si>
+  <si>
+    <t>E. Soulas Moreno</t>
+  </si>
+  <si>
+    <t>Original Authors</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1140,11 +1130,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1152,21 +1141,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1499,7 +1480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}">
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.42578125" style="1" customWidth="1"/>
@@ -1508,10 +1489,11 @@
     <col min="5" max="5" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="28.140625" customWidth="1"/>
     <col min="7" max="7" width="51.140625" customWidth="1"/>
-    <col min="8" max="8" width="39.140625" customWidth="1"/>
+    <col min="8" max="8" width="24.28515625" customWidth="1"/>
+    <col min="9" max="9" width="39.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -1534,71 +1516,80 @@
         <v>12</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:11" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>2013</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>2009</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="G3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>77</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1607,929 +1598,1037 @@
       <c r="E4" s="1">
         <v>2014</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>2019</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="G5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>2024</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="G6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>2021</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="G7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:11" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="1">
         <v>2018</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="1">
         <v>2019</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="1">
         <v>2023</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="1">
         <v>2024</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="1">
         <v>2022</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="G12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="1">
         <v>2022</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="G13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="G13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="1">
         <v>2022</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="G14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="1">
         <v>2013</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="G15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="1">
         <v>2023</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="G16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <v>2021</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="G17" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="G17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="1">
         <v>2016</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="G18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="1">
         <v>2007</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="G19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I19" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="1">
         <v>2022</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="G20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I20" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="1">
         <v>2012</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G21" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="G21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="1">
         <v>2009</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
+      <c r="G22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="1">
         <v>2009</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="G23" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="G23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="1">
         <v>2017</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" t="s">
+      <c r="G24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="1">
         <v>2017</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="G25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="1">
         <v>2023</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="G26" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="G26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="1">
         <v>2024</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
+      <c r="G27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I27" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="1">
         <v>2025</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="G28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="1">
         <v>2016</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G29" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="G29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I29" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <v>2025</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="G30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <v>2022</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="G31" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" t="s">
+      <c r="G31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="1">
         <v>2008</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" t="s">
+      <c r="G32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I32" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="1">
         <v>2016</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="G33" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="G33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I33" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="1">
         <v>2017</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" t="s">
+      <c r="G34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I34" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="1">
         <v>2017</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="G35" t="s">
-        <v>15</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="G35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I35" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="1">
         <v>2021</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" t="s">
+      <c r="G36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I36" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="1">
         <v>2020</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G37" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="G37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="1">
         <v>2020</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G38" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="G38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I38" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="1">
         <v>2012</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="G39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="G39" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I39" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>198</v>
       </c>
@@ -2552,40 +2651,46 @@
         <v>15</v>
       </c>
       <c r="H40" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I40" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I40" s="1"/>
       <c r="J40" s="1"/>
-    </row>
-    <row r="41" spans="1:10" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A41" s="7" t="s">
+      <c r="K40" s="1"/>
+    </row>
+    <row r="41" spans="1:11" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E41" s="7">
+      <c r="E41" s="1">
         <v>2017</v>
       </c>
-      <c r="F41" s="7" t="s">
+      <c r="F41" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="G41" s="7" t="s">
+      <c r="G41" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="H41" s="7" t="s">
+      <c r="H41" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I41" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I41" s="7"/>
-      <c r="J41" s="7"/>
-    </row>
-    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+    </row>
+    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>210</v>
       </c>
@@ -2608,12 +2713,15 @@
         <v>15</v>
       </c>
       <c r="H42" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I42" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I42" s="1"/>
       <c r="J42" s="1"/>
-    </row>
-    <row r="43" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K42" s="1"/>
+    </row>
+    <row r="43" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>212</v>
       </c>
@@ -2636,12 +2744,15 @@
         <v>15</v>
       </c>
       <c r="H43" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I43" s="1"/>
       <c r="J43" s="1"/>
-    </row>
-    <row r="44" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="K43" s="1"/>
+    </row>
+    <row r="44" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>218</v>
       </c>
@@ -2664,12 +2775,15 @@
         <v>15</v>
       </c>
       <c r="H44" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I44" s="1"/>
       <c r="J44" s="1"/>
-    </row>
-    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K44" s="1"/>
+    </row>
+    <row r="45" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>222</v>
       </c>
@@ -2692,12 +2806,15 @@
         <v>15</v>
       </c>
       <c r="H45" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I45" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I45" s="1"/>
       <c r="J45" s="1"/>
-    </row>
-    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K45" s="1"/>
+    </row>
+    <row r="46" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>225</v>
       </c>
@@ -2720,12 +2837,15 @@
         <v>15</v>
       </c>
       <c r="H46" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I46" s="1"/>
       <c r="J46" s="1"/>
-    </row>
-    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K46" s="1"/>
+    </row>
+    <row r="47" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>231</v>
       </c>
@@ -2748,12 +2868,15 @@
         <v>15</v>
       </c>
       <c r="H47" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I47" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I47" s="1"/>
       <c r="J47" s="1"/>
-    </row>
-    <row r="48" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K47" s="1"/>
+    </row>
+    <row r="48" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>235</v>
       </c>
@@ -2776,12 +2899,15 @@
         <v>240</v>
       </c>
       <c r="H48" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I48" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I48" s="1"/>
       <c r="J48" s="1"/>
-    </row>
-    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K48" s="1"/>
+    </row>
+    <row r="49" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>241</v>
       </c>
@@ -2804,12 +2930,15 @@
         <v>15</v>
       </c>
       <c r="H49" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I49" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="I49" s="1"/>
       <c r="J49" s="1"/>
-    </row>
-    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K49" s="1"/>
+    </row>
+    <row r="50" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>250</v>
       </c>
@@ -2832,10 +2961,13 @@
         <v>15</v>
       </c>
       <c r="H50" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I50" s="1" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>251</v>
       </c>
@@ -2858,10 +2990,13 @@
         <v>15</v>
       </c>
       <c r="H51" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I51" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>257</v>
       </c>
@@ -2884,10 +3019,13 @@
         <v>15</v>
       </c>
       <c r="H52" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I52" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>261</v>
       </c>
@@ -2910,10 +3048,13 @@
         <v>15</v>
       </c>
       <c r="H53" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I53" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>267</v>
       </c>
@@ -2936,10 +3077,13 @@
         <v>15</v>
       </c>
       <c r="H54" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I54" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>273</v>
       </c>
@@ -2962,10 +3106,13 @@
         <v>15</v>
       </c>
       <c r="H55" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I55" s="1" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>279</v>
       </c>
@@ -2988,10 +3135,13 @@
         <v>15</v>
       </c>
       <c r="H56" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I56" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>283</v>
       </c>
@@ -3014,10 +3164,13 @@
         <v>15</v>
       </c>
       <c r="H57" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I57" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>287</v>
       </c>
@@ -3040,10 +3193,13 @@
         <v>15</v>
       </c>
       <c r="H58" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I58" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>294</v>
       </c>
@@ -3066,10 +3222,13 @@
         <v>15</v>
       </c>
       <c r="H59" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I59" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>297</v>
       </c>
@@ -3092,10 +3251,13 @@
         <v>15</v>
       </c>
       <c r="H60" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I60" s="1" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>304</v>
       </c>
@@ -3118,10 +3280,13 @@
         <v>15</v>
       </c>
       <c r="H61" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I61" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>308</v>
       </c>
@@ -3144,10 +3309,13 @@
         <v>15</v>
       </c>
       <c r="H62" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I62" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>314</v>
       </c>
@@ -3170,10 +3338,13 @@
         <v>15</v>
       </c>
       <c r="H63" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I63" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>320</v>
       </c>
@@ -3196,10 +3367,13 @@
         <v>15</v>
       </c>
       <c r="H64" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I64" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>325</v>
       </c>
@@ -3222,10 +3396,13 @@
         <v>15</v>
       </c>
       <c r="H65" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I65" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>329</v>
       </c>
@@ -3248,12 +3425,15 @@
         <v>15</v>
       </c>
       <c r="H66" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I66" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I66" s="1"/>
       <c r="J66" s="1"/>
-    </row>
-    <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K66" s="1"/>
+    </row>
+    <row r="67" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>334</v>
       </c>
@@ -3276,14 +3456,17 @@
         <v>338</v>
       </c>
       <c r="H67" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I67" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="H73" s="6"/>
+    <row r="73" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="I73" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>
+  <autoFilter ref="A1:I1" xr:uid="{1BFBE41A-6740-404D-B2B2-771C6F3F6D93}"/>
   <hyperlinks>
     <hyperlink ref="C5" r:id="rId1" xr:uid="{BF75ABFC-35CB-4451-967F-A1889D76545E}"/>
     <hyperlink ref="C13" r:id="rId2" xr:uid="{A86D4BF3-9A8F-4A1A-ACF9-AF107036B055}"/>

</xml_diff>